<commit_message>
Fail the inset checks when a checked element is missing
The card-edge checks dropped missing or hidden elements, so renaming or hiding
an id would have let them pass vacuously. Report such elements as failures and
declare the download locals plainly. Refresh the evidence from a rerun: 115 of
115 on this tree and 70 of 115 on 802cc4a, unchanged in distribution.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidence/s03c4/browser_visual/download.xlsx
+++ b/evidence/s03c4/browser_visual/download.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>089af204cb655eeb0b6adf7c62a20db6</t>
+    <t>24ee76fb7b67582ec6e45bbddc4fd697</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>2a766f7b060b47c7d550d0f114e029f5</t>
+    <t>bc82629005e6850939a619b392bd85d8</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-26T21:08:20-06:00</t>
+    <t>2026-10-26T21:13:50-06:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>

<commit_message>
Refresh acceptance evidence for 173 checks and record the independent review
Rerun on the container-query commit: 173 of 173 checks pass on this tree and 90
of 173 on 802cc4a, which fails every defect category with 83 checks. The
browser report now carries the user agent and the served file hashes, which
equal the committed files. The regression logs are taken on a clean tree, name
the commit under test and end in their exit codes.

Rewrite the acceptance record for the seven viewports and the checks that
assert each defect, and add docs/CODE_REVIEW_S03C4_1.md with both review rounds
and the disposition of each finding, including what no third reviewer saw.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidence/s03c4/browser_visual/download.xlsx
+++ b/evidence/s03c4/browser_visual/download.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>24ee76fb7b67582ec6e45bbddc4fd697</t>
+    <t>45303e46829cc7142295cc468e4835f1</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>bc82629005e6850939a619b392bd85d8</t>
+    <t>6608392d539f63c0d2ab87134a731439</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-26T21:13:50-06:00</t>
+    <t>2026-10-26T21:22:43-06:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>